<commit_message>
docs(sprint-2): encabezados del plan de pruebas en gris claro
</commit_message>
<xml_diff>
--- a/deliverables/sprint-2/Entregable-B-Plan-de-Pruebas-Sprint2.xlsx
+++ b/deliverables/sprint-2/Entregable-B-Plan-de-Pruebas-Sprint2.xlsx
@@ -186,7 +186,7 @@
       <sz val="9"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -208,6 +208,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FF000000"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFD9D9D9"/>
       </patternFill>
     </fill>
   </fills>
@@ -259,7 +264,7 @@
     <xf numFmtId="42" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="44">
+  <cellXfs count="45">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
@@ -387,6 +392,9 @@
     </xf>
     <xf numFmtId="0" fontId="24" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="6">
@@ -902,72 +910,72 @@
       <c r="N5" s="25" t="n"/>
     </row>
     <row r="6" ht="48" customHeight="1" s="26">
-      <c r="A6" s="31" t="inlineStr">
+      <c r="A6" s="44" t="inlineStr">
         <is>
           <t>identificador de test</t>
         </is>
       </c>
-      <c r="B6" s="31" t="inlineStr">
+      <c r="B6" s="44" t="inlineStr">
         <is>
           <t>tipo (unitario, de integracion,  del sistema …)</t>
         </is>
       </c>
-      <c r="C6" s="31" t="inlineStr">
+      <c r="C6" s="44" t="inlineStr">
         <is>
           <t>responsable</t>
         </is>
       </c>
-      <c r="D6" s="31" t="inlineStr">
+      <c r="D6" s="44" t="inlineStr">
         <is>
           <t xml:space="preserve">descripcion </t>
         </is>
       </c>
-      <c r="E6" s="31" t="inlineStr">
+      <c r="E6" s="44" t="inlineStr">
         <is>
           <t>Origen del codigo: Nombre de la funcion/metodo/modulo/programa/clase</t>
         </is>
       </c>
-      <c r="F6" s="31" t="inlineStr">
+      <c r="F6" s="44" t="inlineStr">
         <is>
           <t>datos de entrada</t>
         </is>
       </c>
-      <c r="G6" s="31" t="inlineStr">
+      <c r="G6" s="44" t="inlineStr">
         <is>
           <t>resultado esperado</t>
         </is>
       </c>
-      <c r="H6" s="31" t="inlineStr">
+      <c r="H6" s="44" t="inlineStr">
         <is>
           <t>resultado obtenido</t>
         </is>
       </c>
-      <c r="I6" s="31" t="inlineStr">
+      <c r="I6" s="44" t="inlineStr">
         <is>
           <t>Pasa SI/No</t>
         </is>
       </c>
-      <c r="J6" s="31" t="inlineStr">
+      <c r="J6" s="44" t="inlineStr">
         <is>
           <t>fecha del test</t>
         </is>
       </c>
-      <c r="K6" s="31" t="inlineStr">
+      <c r="K6" s="44" t="inlineStr">
         <is>
           <t>Siguiente paso</t>
         </is>
       </c>
-      <c r="L6" s="31" t="inlineStr">
+      <c r="L6" s="44" t="inlineStr">
         <is>
           <t>Ámbito</t>
         </is>
       </c>
-      <c r="M6" s="31" t="inlineStr">
+      <c r="M6" s="44" t="inlineStr">
         <is>
           <t>Trazabilidad (RF / RNF / RN / historia)</t>
         </is>
       </c>
-      <c r="N6" s="31" t="inlineStr">
+      <c r="N6" s="44" t="inlineStr">
         <is>
           <t>Sprint</t>
         </is>
@@ -8066,37 +8074,37 @@
       <c r="G4" s="25" t="n"/>
     </row>
     <row r="5" ht="23.85" customHeight="1" s="26">
-      <c r="A5" s="31" t="inlineStr">
+      <c r="A5" s="44" t="inlineStr">
         <is>
           <t>Módulo</t>
         </is>
       </c>
-      <c r="B5" s="31" t="inlineStr">
+      <c r="B5" s="44" t="inlineStr">
         <is>
           <t>Casos</t>
         </is>
       </c>
-      <c r="C5" s="31" t="inlineStr">
+      <c r="C5" s="44" t="inlineStr">
         <is>
           <t>Ejecutados</t>
         </is>
       </c>
-      <c r="D5" s="31" t="inlineStr">
+      <c r="D5" s="44" t="inlineStr">
         <is>
           <t>Pasan (SI)</t>
         </is>
       </c>
-      <c r="E5" s="31" t="inlineStr">
+      <c r="E5" s="44" t="inlineStr">
         <is>
           <t>Fallan (NO)</t>
         </is>
       </c>
-      <c r="F5" s="31" t="inlineStr">
+      <c r="F5" s="44" t="inlineStr">
         <is>
           <t>Pendientes</t>
         </is>
       </c>
-      <c r="G5" s="31" t="inlineStr">
+      <c r="G5" s="44" t="inlineStr">
         <is>
           <t>% que pasa de los ejecutados</t>
         </is>
@@ -8497,37 +8505,37 @@
       <c r="G19" s="25" t="n"/>
     </row>
     <row r="20" ht="23.85" customHeight="1" s="26">
-      <c r="A20" s="31" t="inlineStr">
+      <c r="A20" s="44" t="inlineStr">
         <is>
           <t>Tipo</t>
         </is>
       </c>
-      <c r="B20" s="31" t="inlineStr">
+      <c r="B20" s="44" t="inlineStr">
         <is>
           <t>Casos</t>
         </is>
       </c>
-      <c r="C20" s="31" t="inlineStr">
+      <c r="C20" s="44" t="inlineStr">
         <is>
           <t>Ejecutados</t>
         </is>
       </c>
-      <c r="D20" s="31" t="inlineStr">
+      <c r="D20" s="44" t="inlineStr">
         <is>
           <t>Pasan (SI)</t>
         </is>
       </c>
-      <c r="E20" s="31" t="inlineStr">
+      <c r="E20" s="44" t="inlineStr">
         <is>
           <t>Fallan (NO)</t>
         </is>
       </c>
-      <c r="F20" s="31" t="inlineStr">
+      <c r="F20" s="44" t="inlineStr">
         <is>
           <t>Pendientes</t>
         </is>
       </c>
-      <c r="G20" s="31" t="inlineStr">
+      <c r="G20" s="44" t="inlineStr">
         <is>
           <t>% que pasa de los ejecutados</t>
         </is>
@@ -8711,37 +8719,37 @@
       <c r="G27" s="25" t="n"/>
     </row>
     <row r="28" ht="23.85" customHeight="1" s="26">
-      <c r="A28" s="31" t="inlineStr">
+      <c r="A28" s="44" t="inlineStr">
         <is>
           <t>Responsable</t>
         </is>
       </c>
-      <c r="B28" s="31" t="inlineStr">
+      <c r="B28" s="44" t="inlineStr">
         <is>
           <t>Casos</t>
         </is>
       </c>
-      <c r="C28" s="31" t="inlineStr">
+      <c r="C28" s="44" t="inlineStr">
         <is>
           <t>Ejecutados</t>
         </is>
       </c>
-      <c r="D28" s="31" t="inlineStr">
+      <c r="D28" s="44" t="inlineStr">
         <is>
           <t>Pasan (SI)</t>
         </is>
       </c>
-      <c r="E28" s="31" t="inlineStr">
+      <c r="E28" s="44" t="inlineStr">
         <is>
           <t>Fallan (NO)</t>
         </is>
       </c>
-      <c r="F28" s="31" t="inlineStr">
+      <c r="F28" s="44" t="inlineStr">
         <is>
           <t>Pendientes</t>
         </is>
       </c>
-      <c r="G28" s="31" t="inlineStr">
+      <c r="G28" s="44" t="inlineStr">
         <is>
           <t>% que pasa de los ejecutados</t>
         </is>
@@ -8894,37 +8902,37 @@
       <c r="G34" s="25" t="n"/>
     </row>
     <row r="35" ht="23.85" customHeight="1" s="26">
-      <c r="A35" s="31" t="inlineStr">
+      <c r="A35" s="44" t="inlineStr">
         <is>
           <t>Ámbito</t>
         </is>
       </c>
-      <c r="B35" s="31" t="inlineStr">
+      <c r="B35" s="44" t="inlineStr">
         <is>
           <t>Casos</t>
         </is>
       </c>
-      <c r="C35" s="31" t="inlineStr">
+      <c r="C35" s="44" t="inlineStr">
         <is>
           <t>Ejecutados</t>
         </is>
       </c>
-      <c r="D35" s="31" t="inlineStr">
+      <c r="D35" s="44" t="inlineStr">
         <is>
           <t>Pasan (SI)</t>
         </is>
       </c>
-      <c r="E35" s="31" t="inlineStr">
+      <c r="E35" s="44" t="inlineStr">
         <is>
           <t>Fallan (NO)</t>
         </is>
       </c>
-      <c r="F35" s="31" t="inlineStr">
+      <c r="F35" s="44" t="inlineStr">
         <is>
           <t>Pendientes</t>
         </is>
       </c>
-      <c r="G35" s="31" t="inlineStr">
+      <c r="G35" s="44" t="inlineStr">
         <is>
           <t>% que pasa de los ejecutados</t>
         </is>
@@ -9082,37 +9090,37 @@
       <c r="G3" s="25" t="n"/>
     </row>
     <row r="4" ht="15" customHeight="1" s="26">
-      <c r="A4" s="31" t="inlineStr">
+      <c r="A4" s="44" t="inlineStr">
         <is>
           <t>ID</t>
         </is>
       </c>
-      <c r="B4" s="31" t="inlineStr">
+      <c r="B4" s="44" t="inlineStr">
         <is>
           <t>Descripción</t>
         </is>
       </c>
-      <c r="C4" s="31" t="inlineStr">
+      <c r="C4" s="44" t="inlineStr">
         <is>
           <t>Casos</t>
         </is>
       </c>
-      <c r="D4" s="31" t="inlineStr">
+      <c r="D4" s="44" t="inlineStr">
         <is>
           <t>Pasan (SI)</t>
         </is>
       </c>
-      <c r="E4" s="31" t="inlineStr">
+      <c r="E4" s="44" t="inlineStr">
         <is>
           <t>Fallan (NO)</t>
         </is>
       </c>
-      <c r="F4" s="31" t="inlineStr">
+      <c r="F4" s="44" t="inlineStr">
         <is>
           <t>Pendientes</t>
         </is>
       </c>
-      <c r="G4" s="31" t="inlineStr">
+      <c r="G4" s="44" t="inlineStr">
         <is>
           <t>Cobertura</t>
         </is>

</xml_diff>